<commit_message>
Expand verified public-domain corpus
</commit_message>
<xml_diff>
--- a/exports/Hindu_Scriptures_and_Commentaries_Directory.xlsx
+++ b/exports/Hindu_Scriptures_and_Commentaries_Directory.xlsx
@@ -2,11 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repositories" sheetId="1" r:id="Rad8ee68f43614d06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scriptures" sheetId="2" r:id="R5cb5e4a8c63a436a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scholars" sheetId="3" r:id="R8e3f5f5032b74f03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rights Guide" sheetId="4" r:id="Re907724e6b2449ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="5" r:id="R9b14a4a36af6445b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repositories" sheetId="1" r:id="R16fd5cd99ea7433f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scriptures" sheetId="2" r:id="R84f208e09f794084"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scholars" sheetId="3" r:id="R5b1881c656b84058"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rights Guide" sheetId="4" r:id="R5b5a87f694eb49f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="5" r:id="R0bf008ffcfd34328"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mirrored Files" sheetId="6" r:id="Rf3a107c73cea40ce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,7 +18,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="9">
+  <x:fonts count="13">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -69,8 +70,31 @@
       <x:color rgb="FF6B4F00"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="9"/>
+      <x:color rgb="FF5B6770"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -100,6 +124,26 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF18324A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2F7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F7FA"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -199,7 +243,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="58">
+  <x:cellXfs count="79">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -328,6 +372,47 @@
     <x:xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -394,6 +479,25 @@
     <x:tableColumn id="2" name="Meaning"/>
     <x:tableColumn id="3" name="Typical reuse"/>
     <x:tableColumn id="4" name="Important warning"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="MirroredFilesTable" displayName="MirroredFilesTable" ref="A4:K33" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="11">
+    <x:tableColumn id="1" name="ID"/>
+    <x:tableColumn id="2" name="Title"/>
+    <x:tableColumn id="3" name="Layer"/>
+    <x:tableColumn id="4" name="Source"/>
+    <x:tableColumn id="5" name="Source URL"/>
+    <x:tableColumn id="6" name="License"/>
+    <x:tableColumn id="7" name="License URL"/>
+    <x:tableColumn id="8" name="Attribution"/>
+    <x:tableColumn id="9" name="Repository destination"/>
+    <x:tableColumn id="10" name="Rights verification"/>
+    <x:tableColumn id="11" name="SHA-256"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -1077,7 +1181,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R781fe0158ffe4118"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d434e349c664ed4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2029,7 +2133,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d27b3b98be64a29"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc9d5beb2b34407d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3077,7 +3181,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb02e6227d80e4510"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1f92e5a15914e83"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3227,7 +3331,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3fa467fcb124905"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1518e767fdf4b24"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3239,33 +3343,37 @@
     <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="76" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="36" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="34" customHeight="1">
+    <x:row r="1" ht="26" customHeight="1">
       <x:c r="A1" s="3" t="str">
         <x:v>Hindu Scriptures &amp; Commentary Directory</x:v>
       </x:c>
       <x:c r="B1" s="3"/>
       <x:c r="C1" s="3"/>
-      <x:c r="D1" s="3"/>
-      <x:c r="E1" s="3"/>
+      <x:c r="D1" s="73" t="str">
+        <x:v>Verified corpus status</x:v>
+      </x:c>
+      <x:c r="E1" s="73"/>
       <x:c r="F1" s="3"/>
       <x:c r="G1" s="3"/>
       <x:c r="H1" s="3"/>
     </x:row>
-    <x:row r="2" ht="34" customHeight="1">
+    <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
         <x:v>Research catalogue prepared 2026-08-09. Built for lawful discovery, comparison and source verification.</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
-      <x:c r="D2" s="7"/>
-      <x:c r="E2" s="7"/>
+      <x:c r="D2" s="75" t="str">
+        <x:v>Edition-specific coverage as of 2026-08-09</x:v>
+      </x:c>
+      <x:c r="E2" s="75"/>
       <x:c r="F2" s="7"/>
       <x:c r="G2" s="7"/>
       <x:c r="H2" s="7"/>
@@ -3277,6 +3385,12 @@
       <x:c r="B4" s="12" t="str">
         <x:v>Records</x:v>
       </x:c>
+      <x:c r="D4" s="77" t="str">
+        <x:v>Measure</x:v>
+      </x:c>
+      <x:c r="E4" s="77" t="str">
+        <x:v>Count</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="24" hidden="0" customHeight="1">
       <x:c r="A5" s="32" t="str">
@@ -3286,6 +3400,12 @@
         <x:f>COUNTA('Repositories'!A5:A200)</x:f>
         <x:v>16</x:v>
       </x:c>
+      <x:c r="D5" s="78" t="str">
+        <x:v>Mirrored files</x:v>
+      </x:c>
+      <x:c r="E5" s="27" t="n">
+        <x:v>29</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="35" t="str">
@@ -3295,6 +3415,12 @@
         <x:f>COUNTA('Scriptures'!A5:A200)</x:f>
         <x:v>27</x:v>
       </x:c>
+      <x:c r="D6" s="78" t="str">
+        <x:v>Catalogue records with coverage</x:v>
+      </x:c>
+      <x:c r="E6" s="27" t="n">
+        <x:v>53</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="35" t="str">
@@ -3304,6 +3430,12 @@
         <x:f>COUNTA('Scholars'!B5:B200)</x:f>
         <x:v>30</x:v>
       </x:c>
+      <x:c r="D7" s="78" t="str">
+        <x:v>Records pending rights/exact edition</x:v>
+      </x:c>
+      <x:c r="E7" s="27" t="n">
+        <x:v>195</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="24" hidden="0" customHeight="1">
       <x:c r="A8" s="38" t="str">
@@ -3312,6 +3444,12 @@
       <x:c r="B8" s="40" t="n">
         <x:f>COUNTA('Rights Guide'!A5:A50)</x:f>
         <x:v>7</x:v>
+      </x:c>
+      <x:c r="D8" s="78" t="str">
+        <x:v>Total requested records</x:v>
+      </x:c>
+      <x:c r="E8" s="27" t="n">
+        <x:v>248</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -3392,7 +3530,1118 @@
     <x:mergeCell ref="A2:H2"/>
     <x:mergeCell ref="A10:H10"/>
     <x:mergeCell ref="A18:H18"/>
+    <x:mergeCell ref="D1:E1"/>
+    <x:mergeCell ref="D2:E2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="46" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="34" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="52" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="48" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="58" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="68" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="59" t="str">
+        <x:v>Verified Mirrored Files</x:v>
+      </x:c>
+      <x:c r="B1" s="59"/>
+      <x:c r="C1" s="59"/>
+      <x:c r="D1" s="59"/>
+      <x:c r="E1" s="59"/>
+      <x:c r="F1" s="59"/>
+      <x:c r="G1" s="59"/>
+      <x:c r="H1" s="59"/>
+      <x:c r="I1" s="59"/>
+      <x:c r="J1" s="59"/>
+      <x:c r="K1" s="59"/>
+    </x:row>
+    <x:row r="2" ht="32" customHeight="1">
+      <x:c r="A2" s="62" t="str">
+        <x:v>Files stored in the public GitHub repository after edition-level rights review. Source and license links are included for auditability.</x:v>
+      </x:c>
+      <x:c r="B2" s="62"/>
+      <x:c r="C2" s="62"/>
+      <x:c r="D2" s="62"/>
+      <x:c r="E2" s="62"/>
+      <x:c r="F2" s="62"/>
+      <x:c r="G2" s="62"/>
+      <x:c r="H2" s="62"/>
+      <x:c r="I2" s="62"/>
+      <x:c r="J2" s="62"/>
+      <x:c r="K2" s="62"/>
+    </x:row>
+    <x:row r="4" ht="30" customHeight="1">
+      <x:c r="A4" s="66" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="B4" s="66" t="str">
+        <x:v>Title</x:v>
+      </x:c>
+      <x:c r="C4" s="66" t="str">
+        <x:v>Layer</x:v>
+      </x:c>
+      <x:c r="D4" s="66" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+      <x:c r="E4" s="66" t="str">
+        <x:v>Source URL</x:v>
+      </x:c>
+      <x:c r="F4" s="66" t="str">
+        <x:v>License</x:v>
+      </x:c>
+      <x:c r="G4" s="66" t="str">
+        <x:v>License URL</x:v>
+      </x:c>
+      <x:c r="H4" s="66" t="str">
+        <x:v>Attribution</x:v>
+      </x:c>
+      <x:c r="I4" s="66" t="str">
+        <x:v>Repository destination</x:v>
+      </x:c>
+      <x:c r="J4" s="66" t="str">
+        <x:v>Rights verification</x:v>
+      </x:c>
+      <x:c r="K4" s="66" t="str">
+        <x:v>SHA-256</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="56" customHeight="1">
+      <x:c r="A5" s="71" t="str">
+        <x:v>ambuda-ramayana</x:v>
+      </x:c>
+      <x:c r="B5" s="71" t="str">
+        <x:v>Valmiki Ramayana</x:v>
+      </x:c>
+      <x:c r="C5" s="71" t="str">
+        <x:v>root-text</x:v>
+      </x:c>
+      <x:c r="D5" s="71" t="str">
+        <x:v>ambuda-dcs</x:v>
+      </x:c>
+      <x:c r="E5" s="71" t="str">
+        <x:v>https://raw.githubusercontent.com/ambuda-org/dcs/main/ramayanam.txt</x:v>
+      </x:c>
+      <x:c r="F5" s="71" t="str">
+        <x:v>CC-BY-4.0</x:v>
+      </x:c>
+      <x:c r="G5" s="71" t="str">
+        <x:v>https://creativecommons.org/licenses/by/4.0/</x:v>
+      </x:c>
+      <x:c r="H5" s="71" t="str">
+        <x:v>Oliver Hellwig, Digital Corpus of Sanskrit (2010-2021); sanitized distribution by Ambuda</x:v>
+      </x:c>
+      <x:c r="I5" s="71" t="str">
+        <x:v>texts/cc-by-4.0/ambuda/ramayanam.txt</x:v>
+      </x:c>
+      <x:c r="J5" s="71" t="str">
+        <x:v>2026-08-09: Ambuda repository README states DCS license CC BY 4.0.</x:v>
+      </x:c>
+      <x:c r="K5" s="71" t="str">
+        <x:v>f8d45c1289b15182867bd0c94d15886f8d8b1b10c4e7fc9a9b6a78fd5142e3b8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="56" customHeight="1">
+      <x:c r="A6" s="70" t="str">
+        <x:v>ambuda-mahabharata</x:v>
+      </x:c>
+      <x:c r="B6" s="70" t="str">
+        <x:v>Mahabharata</x:v>
+      </x:c>
+      <x:c r="C6" s="70" t="str">
+        <x:v>root-text</x:v>
+      </x:c>
+      <x:c r="D6" s="70" t="str">
+        <x:v>ambuda-dcs</x:v>
+      </x:c>
+      <x:c r="E6" s="70" t="str">
+        <x:v>https://raw.githubusercontent.com/ambuda-org/dcs/main/mahabharatam.txt</x:v>
+      </x:c>
+      <x:c r="F6" s="70" t="str">
+        <x:v>CC-BY-4.0</x:v>
+      </x:c>
+      <x:c r="G6" s="70" t="str">
+        <x:v>https://creativecommons.org/licenses/by/4.0/</x:v>
+      </x:c>
+      <x:c r="H6" s="70" t="str">
+        <x:v>Oliver Hellwig, Digital Corpus of Sanskrit (2010-2021); sanitized distribution by Ambuda</x:v>
+      </x:c>
+      <x:c r="I6" s="70" t="str">
+        <x:v>texts/cc-by-4.0/ambuda/mahabharatam.txt</x:v>
+      </x:c>
+      <x:c r="J6" s="70" t="str">
+        <x:v>2026-08-09: Ambuda repository README states DCS license CC BY 4.0.</x:v>
+      </x:c>
+      <x:c r="K6" s="70" t="str">
+        <x:v>8e871cc252997c03bfb59d47bcfe017c6194041914746cb0a72e4150bd0f120e</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="56" customHeight="1">
+      <x:c r="A7" s="71" t="str">
+        <x:v>sarit-nyaya-vatsyayana</x:v>
+      </x:c>
+      <x:c r="B7" s="71" t="str">
+        <x:v>Nyayasutra with Vatsyayana Nyayabhasya</x:v>
+      </x:c>
+      <x:c r="C7" s="71" t="str">
+        <x:v>root-text-and-commentary</x:v>
+      </x:c>
+      <x:c r="D7" s="71" t="str">
+        <x:v>sarit</x:v>
+      </x:c>
+      <x:c r="E7" s="71" t="str">
+        <x:v>https://raw.githubusercontent.com/sarit/SARIT-corpus/master/vatsyayana-nyayabhasya.xml</x:v>
+      </x:c>
+      <x:c r="F7" s="71" t="str">
+        <x:v>CC-BY-SA-3.0</x:v>
+      </x:c>
+      <x:c r="G7" s="71" t="str">
+        <x:v>https://creativecommons.org/licenses/by-sa/3.0/</x:v>
+      </x:c>
+      <x:c r="H7" s="71" t="str">
+        <x:v>Young Buddhist Association of the University of Tokyo (Bussei); distributed by SARIT</x:v>
+      </x:c>
+      <x:c r="I7" s="71" t="str">
+        <x:v>texts/cc-by-sa-3.0/sarit/vatsyayana-nyayabhasya.xml</x:v>
+      </x:c>
+      <x:c r="J7" s="71" t="str">
+        <x:v>2026-08-09: TEI header explicitly states CC BY-SA 3.0 and attribution.</x:v>
+      </x:c>
+      <x:c r="K7" s="71" t="str">
+        <x:v>f46b12b0b9cf00b8004498a9d6a1433f64b9f3dc1447aa58646398c5739bb3ba</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="56" customHeight="1">
+      <x:c r="A8" s="70" t="str">
+        <x:v>sarit-patanjali-vyasa</x:v>
+      </x:c>
+      <x:c r="B8" s="70" t="str">
+        <x:v>Patanjalayogasastra (Yogasutra with Bhasya)</x:v>
+      </x:c>
+      <x:c r="C8" s="70" t="str">
+        <x:v>root-text-and-commentary</x:v>
+      </x:c>
+      <x:c r="D8" s="70" t="str">
+        <x:v>sarit</x:v>
+      </x:c>
+      <x:c r="E8" s="70" t="str">
+        <x:v>https://raw.githubusercontent.com/sarit/SARIT-corpus/master/patanjalayogasastra.xml</x:v>
+      </x:c>
+      <x:c r="F8" s="70" t="str">
+        <x:v>CC-BY-SA-3.0</x:v>
+      </x:c>
+      <x:c r="G8" s="70" t="str">
+        <x:v>https://creativecommons.org/licenses/by-sa/3.0/</x:v>
+      </x:c>
+      <x:c r="H8" s="70" t="str">
+        <x:v>Philipp Maas; subsequent contributors recorded in TEI revision history; distributed by SARIT</x:v>
+      </x:c>
+      <x:c r="I8" s="70" t="str">
+        <x:v>texts/cc-by-sa-3.0/sarit/patanjalayogasastra.xml</x:v>
+      </x:c>
+      <x:c r="J8" s="70" t="str">
+        <x:v>2026-08-09: TEI header explicitly states CC BY-SA 3.0 and attribution.</x:v>
+      </x:c>
+      <x:c r="K8" s="70" t="str">
+        <x:v>50805a578d250dccbb9a26112d26bdd04115cc895d01509da59d9b8bf7c2e9a6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="56" customHeight="1">
+      <x:c r="A9" s="71" t="str">
+        <x:v>sarit-bhoja-rajamartanda</x:v>
+      </x:c>
+      <x:c r="B9" s="71" t="str">
+        <x:v>Rajamartanda or Bhojavritti</x:v>
+      </x:c>
+      <x:c r="C9" s="71" t="str">
+        <x:v>commentary</x:v>
+      </x:c>
+      <x:c r="D9" s="71" t="str">
+        <x:v>sarit</x:v>
+      </x:c>
+      <x:c r="E9" s="71" t="str">
+        <x:v>https://raw.githubusercontent.com/sarit/SARIT-corpus/master/bhoja-rajamartanda.xml</x:v>
+      </x:c>
+      <x:c r="F9" s="71" t="str">
+        <x:v>CC-BY-SA-3.0</x:v>
+      </x:c>
+      <x:c r="G9" s="71" t="str">
+        <x:v>https://creativecommons.org/licenses/by-sa/3.0/</x:v>
+      </x:c>
+      <x:c r="H9" s="71" t="str">
+        <x:v>Bhojaraja; machine-readable version by Suryansu Ray; distributed by SARIT</x:v>
+      </x:c>
+      <x:c r="I9" s="71" t="str">
+        <x:v>texts/cc-by-sa-3.0/sarit/bhoja-rajamartanda.xml</x:v>
+      </x:c>
+      <x:c r="J9" s="71" t="str">
+        <x:v>2026-08-09: TEI header explicitly licenses the file CC BY-SA 3.0.</x:v>
+      </x:c>
+      <x:c r="K9" s="71" t="str">
+        <x:v>5807ffb3b0d709ed3f87bca3f58f0fc0f410c915752f959db574283cf6a000af</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="56" customHeight="1">
+      <x:c r="A10" s="70" t="str">
+        <x:v>sarit-brahmapurana</x:v>
+      </x:c>
+      <x:c r="B10" s="70" t="str">
+        <x:v>Brahmapurana</x:v>
+      </x:c>
+      <x:c r="C10" s="70" t="str">
+        <x:v>root-text</x:v>
+      </x:c>
+      <x:c r="D10" s="70" t="str">
+        <x:v>sarit</x:v>
+      </x:c>
+      <x:c r="E10" s="70" t="str">
+        <x:v>https://raw.githubusercontent.com/sarit/SARIT-corpus/master/brahmapurana.xml</x:v>
+      </x:c>
+      <x:c r="F10" s="70" t="str">
+        <x:v>CC-BY-SA-3.0</x:v>
+      </x:c>
+      <x:c r="G10" s="70" t="str">
+        <x:v>https://creativecommons.org/licenses/by-sa/3.0/</x:v>
+      </x:c>
+      <x:c r="H10" s="70" t="str">
+        <x:v>Peter Schreiner and Renate Sohnen; SARIT contributors recorded in the TEI header</x:v>
+      </x:c>
+      <x:c r="I10" s="70" t="str">
+        <x:v>texts/cc-by-sa-3.0/sarit/brahmapurana.xml</x:v>
+      </x:c>
+      <x:c r="J10" s="70" t="str">
+        <x:v>2026-08-09: TEI header explicitly licenses the file CC BY-SA 3.0.</x:v>
+      </x:c>
+      <x:c r="K10" s="70" t="str">
+        <x:v>6f4438f5d6ce9c3aa9c12f05fbdeb9485b4f08d68c7b6fbccfe58dcbdd6e5a0b</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="56" customHeight="1">
+      <x:c r="A11" s="71" t="str">
+        <x:v>sarit-carakasamhita</x:v>
+      </x:c>
+      <x:c r="B11" s="71" t="str">
+        <x:v>Carakasamhita with Ayurvedadipika</x:v>
+      </x:c>
+      <x:c r="C11" s="71" t="str">
+        <x:v>root-text-and-commentary</x:v>
+      </x:c>
+      <x:c r="D11" s="71" t="str">
+        <x:v>sarit</x:v>
+      </x:c>
+      <x:c r="E11" s="71" t="str">
+        <x:v>https://raw.githubusercontent.com/sarit/SARIT-corpus/master/carakasamhita.xml</x:v>
+      </x:c>
+      <x:c r="F11" s="71" t="str">
+        <x:v>CC-BY-SA-3.0</x:v>
+      </x:c>
+      <x:c r="G11" s="71" t="str">
+        <x:v>https://creativecommons.org/licenses/by-sa/3.0/</x:v>
+      </x:c>
+      <x:c r="H11" s="71" t="str">
+        <x:v>Tsutomu Yamashita, Yasutaka Muroya, and contributors recorded in the TEI header; distributed by SARIT</x:v>
+      </x:c>
+      <x:c r="I11" s="71" t="str">
+        <x:v>texts/cc-by-sa-3.0/sarit/carakasamhita.xml</x:v>
+      </x:c>
+      <x:c r="J11" s="71" t="str">
+        <x:v>2026-08-09: TEI header explicitly licenses the file CC BY-SA 3.0.</x:v>
+      </x:c>
+      <x:c r="K11" s="71" t="str">
+        <x:v>9f8c1730ff16265b909236539eebcfaa6ddb365fb67c0e07ff4d406b1b583c71</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="56" customHeight="1">
+      <x:c r="A12" s="70" t="str">
+        <x:v>sarit-kautalyarthasastra</x:v>
+      </x:c>
+      <x:c r="B12" s="70" t="str">
+        <x:v>Kautilya Arthasastra</x:v>
+      </x:c>
+      <x:c r="C12" s="70" t="str">
+        <x:v>root-text</x:v>
+      </x:c>
+      <x:c r="D12" s="70" t="str">
+        <x:v>sarit</x:v>
+      </x:c>
+      <x:c r="E12" s="70" t="str">
+        <x:v>https://raw.githubusercontent.com/sarit/SARIT-corpus/master/kautalyarthasastra.xml</x:v>
+      </x:c>
+      <x:c r="F12" s="70" t="str">
+        <x:v>CC-BY-SA-3.0</x:v>
+      </x:c>
+      <x:c r="G12" s="70" t="str">
+        <x:v>https://creativecommons.org/licenses/by-sa/3.0/</x:v>
+      </x:c>
+      <x:c r="H12" s="70" t="str">
+        <x:v>Muneo Tokunaga, Richard Mahoney, Jinkyoung Choi, and SARIT</x:v>
+      </x:c>
+      <x:c r="I12" s="70" t="str">
+        <x:v>texts/cc-by-sa-3.0/sarit/kautalyarthasastra.xml</x:v>
+      </x:c>
+      <x:c r="J12" s="70" t="str">
+        <x:v>2026-08-09: TEI header explicitly licenses the file CC BY-SA 3.0.</x:v>
+      </x:c>
+      <x:c r="K12" s="70" t="str">
+        <x:v>9eed724dd0bc803e9d32fb8032aa432c352f53d0bb5355fb22a8767d7415e1d2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="56" customHeight="1">
+      <x:c r="A13" s="71" t="str">
+        <x:v>sarit-manusmrti</x:v>
+      </x:c>
+      <x:c r="B13" s="71" t="str">
+        <x:v>Manusmrti</x:v>
+      </x:c>
+      <x:c r="C13" s="71" t="str">
+        <x:v>root-text</x:v>
+      </x:c>
+      <x:c r="D13" s="71" t="str">
+        <x:v>sarit</x:v>
+      </x:c>
+      <x:c r="E13" s="71" t="str">
+        <x:v>https://raw.githubusercontent.com/sarit/SARIT-corpus/master/manusmrti.xml</x:v>
+      </x:c>
+      <x:c r="F13" s="71" t="str">
+        <x:v>CC-BY-SA-3.0</x:v>
+      </x:c>
+      <x:c r="G13" s="71" t="str">
+        <x:v>https://creativecommons.org/licenses/by-sa/3.0/</x:v>
+      </x:c>
+      <x:c r="H13" s="71" t="str">
+        <x:v>Contributors and source editions recorded in the TEI header; distributed by SARIT</x:v>
+      </x:c>
+      <x:c r="I13" s="71" t="str">
+        <x:v>texts/cc-by-sa-3.0/sarit/manusmrti.xml</x:v>
+      </x:c>
+      <x:c r="J13" s="71" t="str">
+        <x:v>2026-08-09: TEI header explicitly licenses the file CC BY-SA 3.0.</x:v>
+      </x:c>
+      <x:c r="K13" s="71" t="str">
+        <x:v>eca7717e1543f60bc0784a02f9a900dc572496e74845a8f51c08aaf0c9490ee3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="56" customHeight="1">
+      <x:c r="A14" s="70" t="str">
+        <x:v>sarit-naradasmrti</x:v>
+      </x:c>
+      <x:c r="B14" s="70" t="str">
+        <x:v>Naradasmrti</x:v>
+      </x:c>
+      <x:c r="C14" s="70" t="str">
+        <x:v>root-text</x:v>
+      </x:c>
+      <x:c r="D14" s="70" t="str">
+        <x:v>sarit</x:v>
+      </x:c>
+      <x:c r="E14" s="70" t="str">
+        <x:v>https://raw.githubusercontent.com/sarit/SARIT-corpus/master/naradasmrti.xml</x:v>
+      </x:c>
+      <x:c r="F14" s="70" t="str">
+        <x:v>CC-BY-SA-3.0</x:v>
+      </x:c>
+      <x:c r="G14" s="70" t="str">
+        <x:v>https://creativecommons.org/licenses/by-sa/3.0/</x:v>
+      </x:c>
+      <x:c r="H14" s="70" t="str">
+        <x:v>Richard W. Lariviere, Yasuke Ikari, and contributors recorded in the TEI header; distributed by SARIT</x:v>
+      </x:c>
+      <x:c r="I14" s="70" t="str">
+        <x:v>texts/cc-by-sa-3.0/sarit/naradasmrti.xml</x:v>
+      </x:c>
+      <x:c r="J14" s="70" t="str">
+        <x:v>2026-08-09: TEI header explicitly licenses the file CC BY-SA 3.0.</x:v>
+      </x:c>
+      <x:c r="K14" s="70" t="str">
+        <x:v>965dc6e3e68c183d700b4afb83de76b4f2b44ffed1a7335f2fd6581230ed9f87</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="56" customHeight="1">
+      <x:c r="A15" s="71" t="str">
+        <x:v>sarit-prasastapada</x:v>
+      </x:c>
+      <x:c r="B15" s="71" t="str">
+        <x:v>Padarthadharmasangraha</x:v>
+      </x:c>
+      <x:c r="C15" s="71" t="str">
+        <x:v>root-text</x:v>
+      </x:c>
+      <x:c r="D15" s="71" t="str">
+        <x:v>sarit</x:v>
+      </x:c>
+      <x:c r="E15" s="71" t="str">
+        <x:v>https://raw.githubusercontent.com/sarit/SARIT-corpus/master/prasastapada-padarthadharmasangraha.xml</x:v>
+      </x:c>
+      <x:c r="F15" s="71" t="str">
+        <x:v>CC-BY-SA-3.0</x:v>
+      </x:c>
+      <x:c r="G15" s="71" t="str">
+        <x:v>https://creativecommons.org/licenses/by-sa/3.0/</x:v>
+      </x:c>
+      <x:c r="H15" s="71" t="str">
+        <x:v>Muneo Tokunaga, Yasutaka Muroya, Dominik Wujastyk, and SARIT</x:v>
+      </x:c>
+      <x:c r="I15" s="71" t="str">
+        <x:v>texts/cc-by-sa-3.0/sarit/prasastapada-padarthadharmasangraha.xml</x:v>
+      </x:c>
+      <x:c r="J15" s="71" t="str">
+        <x:v>2026-08-09: TEI header explicitly licenses the file CC BY-SA 3.0.</x:v>
+      </x:c>
+      <x:c r="K15" s="71" t="str">
+        <x:v>bc93f626f56965872dcb33f53294329505b08c10a344e16a5cddba4ddcaebf31</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="56" customHeight="1">
+      <x:c r="A16" s="70" t="str">
+        <x:v>sarit-susrutasamhita</x:v>
+      </x:c>
+      <x:c r="B16" s="70" t="str">
+        <x:v>Susrutasamhita with classical commentaries</x:v>
+      </x:c>
+      <x:c r="C16" s="70" t="str">
+        <x:v>root-text-and-commentary</x:v>
+      </x:c>
+      <x:c r="D16" s="70" t="str">
+        <x:v>sarit</x:v>
+      </x:c>
+      <x:c r="E16" s="70" t="str">
+        <x:v>https://raw.githubusercontent.com/sarit/SARIT-corpus/master/susrutasamhita.xml</x:v>
+      </x:c>
+      <x:c r="F16" s="70" t="str">
+        <x:v>CC-BY-SA-3.0</x:v>
+      </x:c>
+      <x:c r="G16" s="70" t="str">
+        <x:v>https://creativecommons.org/licenses/by-sa/3.0/</x:v>
+      </x:c>
+      <x:c r="H16" s="70" t="str">
+        <x:v>Tsutomu Yamashita, Yasutaka Muroya, and contributors recorded in the TEI header; distributed by SARIT</x:v>
+      </x:c>
+      <x:c r="I16" s="70" t="str">
+        <x:v>texts/cc-by-sa-3.0/sarit/susrutasamhita.xml</x:v>
+      </x:c>
+      <x:c r="J16" s="70" t="str">
+        <x:v>2026-08-09: TEI header explicitly licenses the file CC BY-SA 3.0.</x:v>
+      </x:c>
+      <x:c r="K16" s="70" t="str">
+        <x:v>d6e7618db94ae665f465e63d9c08a1cc1d5358a9f07f58cc5b079e53388c1002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="56" customHeight="1">
+      <x:c r="A17" s="71" t="str">
+        <x:v>sarit-vacaspati-tattvavaisaradi</x:v>
+      </x:c>
+      <x:c r="B17" s="71" t="str">
+        <x:v>Yogasutra with Tattvavaisaradi</x:v>
+      </x:c>
+      <x:c r="C17" s="71" t="str">
+        <x:v>root-text-and-commentary</x:v>
+      </x:c>
+      <x:c r="D17" s="71" t="str">
+        <x:v>sarit</x:v>
+      </x:c>
+      <x:c r="E17" s="71" t="str">
+        <x:v>https://raw.githubusercontent.com/sarit/SARIT-corpus/master/vacaspati-tattvavaisaradi.xml</x:v>
+      </x:c>
+      <x:c r="F17" s="71" t="str">
+        <x:v>CC-BY-SA-3.0</x:v>
+      </x:c>
+      <x:c r="G17" s="71" t="str">
+        <x:v>https://creativecommons.org/licenses/by-sa/3.0/</x:v>
+      </x:c>
+      <x:c r="H17" s="71" t="str">
+        <x:v>Young Buddhist Association of the University of Tokyo (Bussei); distributed by SARIT</x:v>
+      </x:c>
+      <x:c r="I17" s="71" t="str">
+        <x:v>texts/cc-by-sa-3.0/sarit/vacaspati-tattvavaisaradi.xml</x:v>
+      </x:c>
+      <x:c r="J17" s="71" t="str">
+        <x:v>2026-08-09: TEI header explicitly licenses the file CC BY-SA 3.0.</x:v>
+      </x:c>
+      <x:c r="K17" s="71" t="str">
+        <x:v>010527d06955f0163729ec2ebfdd52251f8ba59aaa50e8b5e03fb76fc3cb1b3c</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="56" customHeight="1">
+      <x:c r="A18" s="70" t="str">
+        <x:v>sarit-kumarila-tantravarttika</x:v>
+      </x:c>
+      <x:c r="B18" s="70" t="str">
+        <x:v>Tantravarttika of Kumarila Bhatta</x:v>
+      </x:c>
+      <x:c r="C18" s="70" t="str">
+        <x:v>commentary</x:v>
+      </x:c>
+      <x:c r="D18" s="70" t="str">
+        <x:v>sarit</x:v>
+      </x:c>
+      <x:c r="E18" s="70" t="str">
+        <x:v>https://raw.githubusercontent.com/sarit/SARIT-corpus/master/kumarila-tantravarttika.xml</x:v>
+      </x:c>
+      <x:c r="F18" s="70" t="str">
+        <x:v>CC-BY-SA-4.0</x:v>
+      </x:c>
+      <x:c r="G18" s="70" t="str">
+        <x:v>https://creativecommons.org/licenses/by-sa/4.0/</x:v>
+      </x:c>
+      <x:c r="H18" s="70" t="str">
+        <x:v>Sheldon Pollock, Andrew Ollett, data-entry and SARIT contributors recorded in the TEI header</x:v>
+      </x:c>
+      <x:c r="I18" s="70" t="str">
+        <x:v>texts/cc-by-sa-4.0/sarit/kumarila-tantravarttika.xml</x:v>
+      </x:c>
+      <x:c r="J18" s="70" t="str">
+        <x:v>2026-08-09: TEI header explicitly licenses the file CC BY-SA 4.0.</x:v>
+      </x:c>
+      <x:c r="K18" s="70" t="str">
+        <x:v>f01645a81b66427244323b5c7e6727b259a3c25b2df575cee041a74342c45875</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="56" customHeight="1">
+      <x:c r="A19" s="71" t="str">
+        <x:v>sarit-skandapurana-1-69</x:v>
+      </x:c>
+      <x:c r="B19" s="71" t="str">
+        <x:v>Skandapurana critical edition chapters 1-69</x:v>
+      </x:c>
+      <x:c r="C19" s="71" t="str">
+        <x:v>partial-critical-edition</x:v>
+      </x:c>
+      <x:c r="D19" s="71" t="str">
+        <x:v>sarit</x:v>
+      </x:c>
+      <x:c r="E19" s="71" t="str">
+        <x:v>https://raw.githubusercontent.com/sarit/SARIT-corpus/master/skandapurana.xml</x:v>
+      </x:c>
+      <x:c r="F19" s="71" t="str">
+        <x:v>CC-BY-SA-4.0</x:v>
+      </x:c>
+      <x:c r="G19" s="71" t="str">
+        <x:v>https://creativecommons.org/licenses/by-sa/4.0/</x:v>
+      </x:c>
+      <x:c r="H19" s="71" t="str">
+        <x:v>Editors and contributors recorded in the TEI header; distributed by SARIT</x:v>
+      </x:c>
+      <x:c r="I19" s="71" t="str">
+        <x:v>texts/cc-by-sa-4.0/sarit/skandapurana-adhyayas-1-69.xml</x:v>
+      </x:c>
+      <x:c r="J19" s="71" t="str">
+        <x:v>2026-08-09: TEI header explicitly licenses the file CC BY-SA 4.0; this is not the whole received Skandapurana.</x:v>
+      </x:c>
+      <x:c r="K19" s="71" t="str">
+        <x:v>28ad61d4867a7515d55c2628bab744ddc78e53afc452ba71ed9abda1fdaad821</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="56" customHeight="1">
+      <x:c r="A20" s="70" t="str">
+        <x:v>sarit-vijnanesvara-mitaksara</x:v>
+      </x:c>
+      <x:c r="B20" s="70" t="str">
+        <x:v>Mitaksara commentary on Yajnavalkya Dharmasastra</x:v>
+      </x:c>
+      <x:c r="C20" s="70" t="str">
+        <x:v>root-text-and-commentary</x:v>
+      </x:c>
+      <x:c r="D20" s="70" t="str">
+        <x:v>sarit</x:v>
+      </x:c>
+      <x:c r="E20" s="70" t="str">
+        <x:v>https://raw.githubusercontent.com/sarit/SARIT-corpus/master/vijnanesvara-mitaksara.xml</x:v>
+      </x:c>
+      <x:c r="F20" s="70" t="str">
+        <x:v>CC-BY-SA-4.0</x:v>
+      </x:c>
+      <x:c r="G20" s="70" t="str">
+        <x:v>https://creativecommons.org/licenses/by-sa/4.0/</x:v>
+      </x:c>
+      <x:c r="H20" s="70" t="str">
+        <x:v>Patrick Olivelle, Donald R. Davis Jr., Amy Hyne-Sutherland, Nikola Rajic, GRETIL, and SARIT</x:v>
+      </x:c>
+      <x:c r="I20" s="70" t="str">
+        <x:v>texts/cc-by-sa-4.0/sarit/vijnanesvara-mitaksara.xml</x:v>
+      </x:c>
+      <x:c r="J20" s="70" t="str">
+        <x:v>2026-08-09: TEI header explicitly licenses the file CC BY-SA 4.0.</x:v>
+      </x:c>
+      <x:c r="K20" s="70" t="str">
+        <x:v>784509084b553d2665be58ac97c80bb4e5a9826efbd73483b247bf7ed4fa346f</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="56" customHeight="1">
+      <x:c r="A21" s="71" t="str">
+        <x:v>pg-2388-bhagavad-gita</x:v>
+      </x:c>
+      <x:c r="B21" s="71" t="str">
+        <x:v>The Song Celestial or Bhagavad-Gita</x:v>
+      </x:c>
+      <x:c r="C21" s="71" t="str">
+        <x:v>english-translation</x:v>
+      </x:c>
+      <x:c r="D21" s="71" t="str">
+        <x:v>project-gutenberg</x:v>
+      </x:c>
+      <x:c r="E21" s="71" t="str">
+        <x:v>https://www.gutenberg.org/cache/epub/2388/pg2388.txt</x:v>
+      </x:c>
+      <x:c r="F21" s="71" t="str">
+        <x:v>Public-Domain-US</x:v>
+      </x:c>
+      <x:c r="G21" s="71" t="str">
+        <x:v>https://www.gutenberg.org/policy/license.html</x:v>
+      </x:c>
+      <x:c r="H21" s="71" t="str">
+        <x:v>Edwin Arnold (translator); Project Gutenberg ebook 2388</x:v>
+      </x:c>
+      <x:c r="I21" s="71" t="str">
+        <x:v>texts/public-domain-us/project-gutenberg/pg2388-bhagavad-gita.txt</x:v>
+      </x:c>
+      <x:c r="J21" s="71" t="str">
+        <x:v>2026-08-09: Project Gutenberg item states public domain in the USA and includes the Project Gutenberg License.</x:v>
+      </x:c>
+      <x:c r="K21" s="71" t="str">
+        <x:v>85b22401a9d256179f9a2e407215eb516da9b8213f23c32e03d66709d839a9e0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="56" customHeight="1">
+      <x:c r="A22" s="70" t="str">
+        <x:v>pg-2526-yoga-sutras</x:v>
+      </x:c>
+      <x:c r="B22" s="70" t="str">
+        <x:v>The Yoga Sutras of Patanjali</x:v>
+      </x:c>
+      <x:c r="C22" s="70" t="str">
+        <x:v>english-translation-and-commentary</x:v>
+      </x:c>
+      <x:c r="D22" s="70" t="str">
+        <x:v>project-gutenberg</x:v>
+      </x:c>
+      <x:c r="E22" s="70" t="str">
+        <x:v>https://www.gutenberg.org/cache/epub/2526/pg2526.txt</x:v>
+      </x:c>
+      <x:c r="F22" s="70" t="str">
+        <x:v>Public-Domain-US</x:v>
+      </x:c>
+      <x:c r="G22" s="70" t="str">
+        <x:v>https://www.gutenberg.org/policy/license.html</x:v>
+      </x:c>
+      <x:c r="H22" s="70" t="str">
+        <x:v>Charles Johnston (editor/translator); Project Gutenberg ebook 2526</x:v>
+      </x:c>
+      <x:c r="I22" s="70" t="str">
+        <x:v>texts/public-domain-us/project-gutenberg/pg2526-yoga-sutras.txt</x:v>
+      </x:c>
+      <x:c r="J22" s="70" t="str">
+        <x:v>2026-08-09: Project Gutenberg item states public domain in the USA and includes the Project Gutenberg License.</x:v>
+      </x:c>
+      <x:c r="K22" s="70" t="str">
+        <x:v>8993f37c71c83095c46f3355aa4c9350838b1043edf443f9653f48cd157e88f5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="56" customHeight="1">
+      <x:c r="A23" s="71" t="str">
+        <x:v>pg-3283-upanishads</x:v>
+      </x:c>
+      <x:c r="B23" s="71" t="str">
+        <x:v>The Upanishads: Isa Katha and Kena</x:v>
+      </x:c>
+      <x:c r="C23" s="71" t="str">
+        <x:v>english-translation-and-commentary</x:v>
+      </x:c>
+      <x:c r="D23" s="71" t="str">
+        <x:v>project-gutenberg</x:v>
+      </x:c>
+      <x:c r="E23" s="71" t="str">
+        <x:v>https://www.gutenberg.org/cache/epub/3283/pg3283.txt</x:v>
+      </x:c>
+      <x:c r="F23" s="71" t="str">
+        <x:v>Public-Domain-US</x:v>
+      </x:c>
+      <x:c r="G23" s="71" t="str">
+        <x:v>https://www.gutenberg.org/policy/license.html</x:v>
+      </x:c>
+      <x:c r="H23" s="71" t="str">
+        <x:v>Swami Paramananda (translator/commentator); Project Gutenberg ebook 3283</x:v>
+      </x:c>
+      <x:c r="I23" s="71" t="str">
+        <x:v>texts/public-domain-us/project-gutenberg/pg3283-upanishads-paramananda.txt</x:v>
+      </x:c>
+      <x:c r="J23" s="71" t="str">
+        <x:v>2026-08-09: Project Gutenberg item states public domain in the USA and includes the Project Gutenberg License.</x:v>
+      </x:c>
+      <x:c r="K23" s="71" t="str">
+        <x:v>2ffc941173d8fd10c16eea7bfb4ab2ace13cf9e734228c71f367402f9236aa46</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="56" customHeight="1">
+      <x:c r="A24" s="70" t="str">
+        <x:v>pg-7297-ramanuja-vedanta-sutras</x:v>
+      </x:c>
+      <x:c r="B24" s="70" t="str">
+        <x:v>The Vedanta-Sutras with Ramanuja's commentary</x:v>
+      </x:c>
+      <x:c r="C24" s="70" t="str">
+        <x:v>english-translation-and-commentary</x:v>
+      </x:c>
+      <x:c r="D24" s="70" t="str">
+        <x:v>project-gutenberg</x:v>
+      </x:c>
+      <x:c r="E24" s="70" t="str">
+        <x:v>https://www.gutenberg.org/cache/epub/7297/pg7297.txt</x:v>
+      </x:c>
+      <x:c r="F24" s="70" t="str">
+        <x:v>Public-Domain-US</x:v>
+      </x:c>
+      <x:c r="G24" s="70" t="str">
+        <x:v>https://www.gutenberg.org/policy/license.html</x:v>
+      </x:c>
+      <x:c r="H24" s="70" t="str">
+        <x:v>George Thibaut (translator), Ramanuja (commentator); Project Gutenberg ebook 7297</x:v>
+      </x:c>
+      <x:c r="I24" s="70" t="str">
+        <x:v>texts/public-domain-us/project-gutenberg/pg7297-vedanta-sutras-ramanuja.txt</x:v>
+      </x:c>
+      <x:c r="J24" s="70" t="str">
+        <x:v>2026-08-09: Project Gutenberg item states public domain in the USA and includes the Project Gutenberg License.</x:v>
+      </x:c>
+      <x:c r="K24" s="70" t="str">
+        <x:v>dde277b01b1ce3b05a88dd168e2c161ae33475be9edd822877b7b301d84b0198</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="56" customHeight="1">
+      <x:c r="A25" s="71" t="str">
+        <x:v>pg-15474-mahabharata-vol-1</x:v>
+      </x:c>
+      <x:c r="B25" s="71" t="str">
+        <x:v>The Mahabharata English prose volume 1 books 1-3</x:v>
+      </x:c>
+      <x:c r="C25" s="71" t="str">
+        <x:v>english-translation</x:v>
+      </x:c>
+      <x:c r="D25" s="71" t="str">
+        <x:v>project-gutenberg</x:v>
+      </x:c>
+      <x:c r="E25" s="71" t="str">
+        <x:v>https://www.gutenberg.org/cache/epub/15474/pg15474.txt</x:v>
+      </x:c>
+      <x:c r="F25" s="71" t="str">
+        <x:v>Public-Domain-US</x:v>
+      </x:c>
+      <x:c r="G25" s="71" t="str">
+        <x:v>https://www.gutenberg.org/policy/license.html</x:v>
+      </x:c>
+      <x:c r="H25" s="71" t="str">
+        <x:v>Kisari Mohan Ganguli (translator); Project Gutenberg ebook 15474</x:v>
+      </x:c>
+      <x:c r="I25" s="71" t="str">
+        <x:v>texts/public-domain-us/project-gutenberg/pg15474-mahabharata-vol-1.txt</x:v>
+      </x:c>
+      <x:c r="J25" s="71" t="str">
+        <x:v>2026-08-09: Project Gutenberg item states public domain in the USA and includes the Project Gutenberg License.</x:v>
+      </x:c>
+      <x:c r="K25" s="71" t="str">
+        <x:v>6936769ca526bc5486335940958f43d036414d2fd29dcc17259610fa95b66b75</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="56" customHeight="1">
+      <x:c r="A26" s="70" t="str">
+        <x:v>pg-15475-mahabharata-vol-2</x:v>
+      </x:c>
+      <x:c r="B26" s="70" t="str">
+        <x:v>The Mahabharata English prose volume 2 books 4-7</x:v>
+      </x:c>
+      <x:c r="C26" s="70" t="str">
+        <x:v>english-translation</x:v>
+      </x:c>
+      <x:c r="D26" s="70" t="str">
+        <x:v>project-gutenberg</x:v>
+      </x:c>
+      <x:c r="E26" s="70" t="str">
+        <x:v>https://www.gutenberg.org/cache/epub/15475/pg15475.txt</x:v>
+      </x:c>
+      <x:c r="F26" s="70" t="str">
+        <x:v>Public-Domain-US</x:v>
+      </x:c>
+      <x:c r="G26" s="70" t="str">
+        <x:v>https://www.gutenberg.org/policy/license.html</x:v>
+      </x:c>
+      <x:c r="H26" s="70" t="str">
+        <x:v>Kisari Mohan Ganguli (translator); Project Gutenberg ebook 15475</x:v>
+      </x:c>
+      <x:c r="I26" s="70" t="str">
+        <x:v>texts/public-domain-us/project-gutenberg/pg15475-mahabharata-vol-2.txt</x:v>
+      </x:c>
+      <x:c r="J26" s="70" t="str">
+        <x:v>2026-08-09: Project Gutenberg item states public domain in the USA and includes the Project Gutenberg License.</x:v>
+      </x:c>
+      <x:c r="K26" s="70" t="str">
+        <x:v>135076505fc86930e9817858def7f1448d73d5dbf6000c841eafcc2e73f59eb3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="56" customHeight="1">
+      <x:c r="A27" s="71" t="str">
+        <x:v>pg-15476-mahabharata-vol-3</x:v>
+      </x:c>
+      <x:c r="B27" s="71" t="str">
+        <x:v>The Mahabharata English prose volume 3 books 8-12</x:v>
+      </x:c>
+      <x:c r="C27" s="71" t="str">
+        <x:v>english-translation</x:v>
+      </x:c>
+      <x:c r="D27" s="71" t="str">
+        <x:v>project-gutenberg</x:v>
+      </x:c>
+      <x:c r="E27" s="71" t="str">
+        <x:v>https://www.gutenberg.org/cache/epub/15476/pg15476.txt</x:v>
+      </x:c>
+      <x:c r="F27" s="71" t="str">
+        <x:v>Public-Domain-US</x:v>
+      </x:c>
+      <x:c r="G27" s="71" t="str">
+        <x:v>https://www.gutenberg.org/policy/license.html</x:v>
+      </x:c>
+      <x:c r="H27" s="71" t="str">
+        <x:v>Kisari Mohan Ganguli (translator); Project Gutenberg ebook 15476</x:v>
+      </x:c>
+      <x:c r="I27" s="71" t="str">
+        <x:v>texts/public-domain-us/project-gutenberg/pg15476-mahabharata-vol-3.txt</x:v>
+      </x:c>
+      <x:c r="J27" s="71" t="str">
+        <x:v>2026-08-09: Project Gutenberg item states public domain in the USA and includes the Project Gutenberg License.</x:v>
+      </x:c>
+      <x:c r="K27" s="71" t="str">
+        <x:v>2d4d53b9c4892ebdc5a4bfa59458d0e0acf9742d3ce0f3b7b1b428ab838f402d</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="56" customHeight="1">
+      <x:c r="A28" s="70" t="str">
+        <x:v>pg-15477-mahabharata-vol-4</x:v>
+      </x:c>
+      <x:c r="B28" s="70" t="str">
+        <x:v>The Mahabharata English prose volume 4 books 13-18</x:v>
+      </x:c>
+      <x:c r="C28" s="70" t="str">
+        <x:v>english-translation</x:v>
+      </x:c>
+      <x:c r="D28" s="70" t="str">
+        <x:v>project-gutenberg</x:v>
+      </x:c>
+      <x:c r="E28" s="70" t="str">
+        <x:v>https://www.gutenberg.org/cache/epub/15477/pg15477.txt</x:v>
+      </x:c>
+      <x:c r="F28" s="70" t="str">
+        <x:v>Public-Domain-US</x:v>
+      </x:c>
+      <x:c r="G28" s="70" t="str">
+        <x:v>https://www.gutenberg.org/policy/license.html</x:v>
+      </x:c>
+      <x:c r="H28" s="70" t="str">
+        <x:v>Kisari Mohan Ganguli (translator); Project Gutenberg ebook 15477</x:v>
+      </x:c>
+      <x:c r="I28" s="70" t="str">
+        <x:v>texts/public-domain-us/project-gutenberg/pg15477-mahabharata-vol-4.txt</x:v>
+      </x:c>
+      <x:c r="J28" s="70" t="str">
+        <x:v>2026-08-09: Project Gutenberg item states public domain in the USA and includes the Project Gutenberg License.</x:v>
+      </x:c>
+      <x:c r="K28" s="70" t="str">
+        <x:v>60de2a2f82f22247fdb72096c7ebbb01b63ad42770506c10f6d7c7a82868e437</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="56" customHeight="1">
+      <x:c r="A29" s="71" t="str">
+        <x:v>pg-16295-shankara-vedanta-sutras</x:v>
+      </x:c>
+      <x:c r="B29" s="71" t="str">
+        <x:v>The Vedanta-Sutras with Shankaracharya's commentary part 1</x:v>
+      </x:c>
+      <x:c r="C29" s="71" t="str">
+        <x:v>english-translation-and-commentary</x:v>
+      </x:c>
+      <x:c r="D29" s="71" t="str">
+        <x:v>project-gutenberg</x:v>
+      </x:c>
+      <x:c r="E29" s="71" t="str">
+        <x:v>https://www.gutenberg.org/cache/epub/16295/pg16295.txt</x:v>
+      </x:c>
+      <x:c r="F29" s="71" t="str">
+        <x:v>Public-Domain-US</x:v>
+      </x:c>
+      <x:c r="G29" s="71" t="str">
+        <x:v>https://www.gutenberg.org/policy/license.html</x:v>
+      </x:c>
+      <x:c r="H29" s="71" t="str">
+        <x:v>George Thibaut (translator), Shankaracharya (commentator); Project Gutenberg ebook 16295</x:v>
+      </x:c>
+      <x:c r="I29" s="71" t="str">
+        <x:v>texts/public-domain-us/project-gutenberg/pg16295-vedanta-sutras-shankara.txt</x:v>
+      </x:c>
+      <x:c r="J29" s="71" t="str">
+        <x:v>2026-08-09: Project Gutenberg item states public domain in the USA and includes the Project Gutenberg License.</x:v>
+      </x:c>
+      <x:c r="K29" s="71" t="str">
+        <x:v>92376bcad34794e1fbaa61b89f3c6681f61c44e4e04973deddd63bbaf78045a1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="56" customHeight="1">
+      <x:c r="A30" s="70" t="str">
+        <x:v>pg-61937-harivamsha</x:v>
+      </x:c>
+      <x:c r="B30" s="70" t="str">
+        <x:v>A Prose English Translation of Harivamsha</x:v>
+      </x:c>
+      <x:c r="C30" s="70" t="str">
+        <x:v>english-translation</x:v>
+      </x:c>
+      <x:c r="D30" s="70" t="str">
+        <x:v>project-gutenberg</x:v>
+      </x:c>
+      <x:c r="E30" s="70" t="str">
+        <x:v>https://www.gutenberg.org/cache/epub/61937/pg61937.txt</x:v>
+      </x:c>
+      <x:c r="F30" s="70" t="str">
+        <x:v>Public-Domain-US</x:v>
+      </x:c>
+      <x:c r="G30" s="70" t="str">
+        <x:v>https://www.gutenberg.org/policy/license.html</x:v>
+      </x:c>
+      <x:c r="H30" s="70" t="str">
+        <x:v>Manmatha Nath Dutt (translator); Project Gutenberg ebook 61937</x:v>
+      </x:c>
+      <x:c r="I30" s="70" t="str">
+        <x:v>texts/public-domain-us/project-gutenberg/pg61937-harivamsha.txt</x:v>
+      </x:c>
+      <x:c r="J30" s="70" t="str">
+        <x:v>2026-08-09: Project Gutenberg item states public domain in the USA and includes the Project Gutenberg License.</x:v>
+      </x:c>
+      <x:c r="K30" s="70" t="str">
+        <x:v>839d1c8e329c3aa9e64d2864f88acf6cd2838d61b1ead5c4aa5ecad1a891f4d6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="56" customHeight="1">
+      <x:c r="A31" s="71" t="str">
+        <x:v>pg-66208-vishnupurana</x:v>
+      </x:c>
+      <x:c r="B31" s="71" t="str">
+        <x:v>A Prose English Translation of Vishnupuranam</x:v>
+      </x:c>
+      <x:c r="C31" s="71" t="str">
+        <x:v>english-translation</x:v>
+      </x:c>
+      <x:c r="D31" s="71" t="str">
+        <x:v>project-gutenberg</x:v>
+      </x:c>
+      <x:c r="E31" s="71" t="str">
+        <x:v>https://www.gutenberg.org/cache/epub/66208/pg66208.txt</x:v>
+      </x:c>
+      <x:c r="F31" s="71" t="str">
+        <x:v>Public-Domain-US</x:v>
+      </x:c>
+      <x:c r="G31" s="71" t="str">
+        <x:v>https://www.gutenberg.org/policy/license.html</x:v>
+      </x:c>
+      <x:c r="H31" s="71" t="str">
+        <x:v>Manmatha Nath Dutt and H. H. Wilson (translators); Project Gutenberg ebook 66208</x:v>
+      </x:c>
+      <x:c r="I31" s="71" t="str">
+        <x:v>texts/public-domain-us/project-gutenberg/pg66208-vishnupuranam.txt</x:v>
+      </x:c>
+      <x:c r="J31" s="71" t="str">
+        <x:v>2026-08-09: Project Gutenberg item states public domain in the USA and includes the Project Gutenberg License.</x:v>
+      </x:c>
+      <x:c r="K31" s="71" t="str">
+        <x:v>924d8c109ddf87a26fab4025556be7b74dbf0c21534e253bfb4561f711956bb5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="56" customHeight="1">
+      <x:c r="A32" s="70" t="str">
+        <x:v>ia-upanishads-sbe-1</x:v>
+      </x:c>
+      <x:c r="B32" s="70" t="str">
+        <x:v>The Upanishads Part I Sacred Books of the East volume 1</x:v>
+      </x:c>
+      <x:c r="C32" s="70" t="str">
+        <x:v>english-translation</x:v>
+      </x:c>
+      <x:c r="D32" s="70" t="str">
+        <x:v>internet-archive</x:v>
+      </x:c>
+      <x:c r="E32" s="70" t="str">
+        <x:v>https://archive.org/download/upanishads01ml/upanishads01ml_djvu.txt</x:v>
+      </x:c>
+      <x:c r="F32" s="70" t="str">
+        <x:v>Public-Domain-US</x:v>
+      </x:c>
+      <x:c r="G32" s="70" t="str">
+        <x:v>https://www.copyright.gov/help/faq/faq-duration.html</x:v>
+      </x:c>
+      <x:c r="H32" s="70" t="str">
+        <x:v>F. Max Muller (translator/editor), Oxford University Press 1879; OCR derivative hosted by Internet Archive</x:v>
+      </x:c>
+      <x:c r="I32" s="70" t="str">
+        <x:v>texts/public-domain-us/internet-archive/upanishads-sbe-vol-1-ocr.txt</x:v>
+      </x:c>
+      <x:c r="J32" s="70" t="str">
+        <x:v>2026-08-09: The underlying 1879 edition is public domain in the United States; OCR quality should be checked against the linked scan.</x:v>
+      </x:c>
+      <x:c r="K32" s="70" t="str">
+        <x:v>e1e8b802db19f2b2f7f60c03be79d2aa16f4b36bb6733c8d54084113b56eb884</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="56" customHeight="1">
+      <x:c r="A33" s="71" t="str">
+        <x:v>ia-upanishads-sbe-15</x:v>
+      </x:c>
+      <x:c r="B33" s="71" t="str">
+        <x:v>The Upanishads Part II Sacred Books of the East volume 15</x:v>
+      </x:c>
+      <x:c r="C33" s="71" t="str">
+        <x:v>english-translation</x:v>
+      </x:c>
+      <x:c r="D33" s="71" t="str">
+        <x:v>internet-archive</x:v>
+      </x:c>
+      <x:c r="E33" s="71" t="str">
+        <x:v>https://archive.org/download/upanishads02ml/upanishads02ml_djvu.txt</x:v>
+      </x:c>
+      <x:c r="F33" s="71" t="str">
+        <x:v>Public-Domain-US</x:v>
+      </x:c>
+      <x:c r="G33" s="71" t="str">
+        <x:v>https://www.copyright.gov/help/faq/faq-duration.html</x:v>
+      </x:c>
+      <x:c r="H33" s="71" t="str">
+        <x:v>F. Max Muller (translator/editor), Oxford University Press 1884; OCR derivative hosted by Internet Archive</x:v>
+      </x:c>
+      <x:c r="I33" s="71" t="str">
+        <x:v>texts/public-domain-us/internet-archive/upanishads-sbe-vol-15-ocr.txt</x:v>
+      </x:c>
+      <x:c r="J33" s="71" t="str">
+        <x:v>2026-08-09: The underlying 1884 edition is public domain in the United States; OCR quality should be checked against the linked scan.</x:v>
+      </x:c>
+      <x:c r="K33" s="71" t="str">
+        <x:v>1f2223b0292eb87368cd5373b684b6335373318097847aa18716cfb119c4d6e3</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:K1"/>
+    <x:mergeCell ref="A2:K2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R779b5744ece64984"/>
+  </x:tableParts>
+</x:worksheet>
 </file>
</xml_diff>